<commit_message>
reformatação  pos recuperação incial
reformatação apos recuperação da lista inicial nao formatada e vazia
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Giovana Mazzei\Faculdade\Business Systems Planning, Analysis &amp; Design\Projetos2SIPG\PastaDocsEngenhariaSw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Giovana Mazzei\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F718C15F-5996-4CF6-A948-96176442F5A8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9828B1DA-AE55-45B5-9130-450632F666AD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10476" windowHeight="5556" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -54,16 +54,57 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="4" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -71,12 +112,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -357,37 +432,190 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.77734375" customWidth="1"/>
-    <col min="2" max="2" width="25.5546875" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="47.6640625" customWidth="1"/>
+    <col min="4" max="4" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
2a versao requisitos de pesquisa de referencia
segunda versao da lista com requisitos identificados por pesquisa de referenicas
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Giovana Mazzei\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9828B1DA-AE55-45B5-9130-450632F666AD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA6D0FC6-8094-4DA8-8A79-52E95F3DD796}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10476" windowHeight="5556" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>LISTA DE REQUISITOS DO PROJETO DE SISTEMA DE INFORMAÇÃO PARA GERENCIAR ESTACIONAMENTOS</t>
   </si>
@@ -40,6 +40,132 @@
   </si>
   <si>
     <t>Descrição da regra de domínio</t>
+  </si>
+  <si>
+    <t>Rf001</t>
+  </si>
+  <si>
+    <t>tarifação inteligente</t>
+  </si>
+  <si>
+    <t>planos mensais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parcerias de convenios </t>
+  </si>
+  <si>
+    <t>Rf002</t>
+  </si>
+  <si>
+    <t>Rf003</t>
+  </si>
+  <si>
+    <t>Rf004</t>
+  </si>
+  <si>
+    <t>acompanhamento do caixa</t>
+  </si>
+  <si>
+    <t>criação de anotaçoes/lembretes</t>
+  </si>
+  <si>
+    <t>criacao de vouchers de desconto</t>
+  </si>
+  <si>
+    <t>controle de serviços extras</t>
+  </si>
+  <si>
+    <t>proteçao do sistema anti-fraude</t>
+  </si>
+  <si>
+    <t>acrescimo de serviço de lava jato, lava rapido, cera, polimento</t>
+  </si>
+  <si>
+    <t>aplicação movel para motoristas acharem estacionamentos com vagas livres na regiao em que estao</t>
+  </si>
+  <si>
+    <t>localizar estacionamentos disponiveis</t>
+  </si>
+  <si>
+    <t>reserva de vagas em tempo real</t>
+  </si>
+  <si>
+    <t>um motorista em movimento ou antes de sair com seu carro pode reservar uma vaga para um dia e horario em um estacionamento</t>
+  </si>
+  <si>
+    <t>pagamento integrado</t>
+  </si>
+  <si>
+    <t>aceitar pagamento de cartao ou pix</t>
+  </si>
+  <si>
+    <t>apresentar um grafico de barros com a quantidade de veiculos por dia de um mês selecionado</t>
+  </si>
+  <si>
+    <t>dashboard/painel de acompanhamento de ocupação por mês</t>
+  </si>
+  <si>
+    <t>apresentar um grafico de linhas cos os meses no eixo x e o valor de montante no eixo y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dashboard/painel de acompanhamento receita mês a mês </t>
+  </si>
+  <si>
+    <t>Rf005</t>
+  </si>
+  <si>
+    <t>Rf006</t>
+  </si>
+  <si>
+    <t>Rf007</t>
+  </si>
+  <si>
+    <t>Rf008</t>
+  </si>
+  <si>
+    <t>Rf009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notificação de tempppo restante </t>
+  </si>
+  <si>
+    <t>Rf010</t>
+  </si>
+  <si>
+    <t>Rf011</t>
+  </si>
+  <si>
+    <t>Rf012</t>
+  </si>
+  <si>
+    <t>com auxilição de ia o sistema vai propror uma tarifa conforme as praticas concorrentes da regiao</t>
+  </si>
+  <si>
+    <t>tabalea de precos exclusiva para mensalistas</t>
+  </si>
+  <si>
+    <t>tabela de precos exclusivapara esyacionamento avulso cobrado conforme dia e hora</t>
+  </si>
+  <si>
+    <t>registro de pagamento com controle fiscal</t>
+  </si>
+  <si>
+    <t>tabela de precos exclusivo para conevniados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gerar automaticamento um voucher de desconto cnformo o numero de hrs q o cliente acumulou em um periodo </t>
+  </si>
+  <si>
+    <t>planos avulsos</t>
+  </si>
+  <si>
+    <t>Rf013</t>
+  </si>
+  <si>
+    <t>Rf014</t>
+  </si>
+  <si>
+    <t>enviar mensagem por wpp para o motorista avisanado o tmepo reestante em caso de fechamneto do estacionamento</t>
   </si>
 </sst>
 </file>
@@ -436,9 +562,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.77734375" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="2" max="2" width="50.88671875" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="56.77734375" customWidth="1"/>
+    <col min="4" max="4" width="97.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -471,100 +597,186 @@
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="D10" s="2" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="D13" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="D16" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="D17" s="2" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="A18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="D18" s="2" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="B19" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>

</xml_diff>